<commit_message>
Fix Catalan UI strings; translate English reading rules for all natives
- ca: Escalfament, Pròxima lliçó, Més difícil, Reprodueix-ho tot,
  Millora el pla, Envia i puntua, Expressió oral, step-3 title, casing
- Reading rules (Правила sheet has only ru/en/es/uk) generated for 15 more
  native languages; reading_app.load() uses them
- Source fixes: truncated lesson 20 rule, IPA typos in lessons 68/75
- Test: every native has rules with IPA intact

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/reading_lessons.xlsx
+++ b/data/reading_lessons.xlsx
@@ -81827,22 +81827,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ii, Yy в бу [ı]: 'funny ['fʌnı]; mini ['mını].</t>
+          <t>Ii, Yy в безударном слоге читаются как [ı]: 'funny ['fʌnı]; mini ['mını].</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ii, Yy in bu [ı]: 'funny ['fʌnı]; mini ['mını].</t>
+          <t>Ii, Yy in an unstressed syllable are pronounced as [ı]: 'funny ['fʌnı]; mini ['mını].</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ii, Yy en bu [ı]: 'funny ['fʌnı]; mini ['mını].</t>
+          <t>Ii, Yy en sílaba átona se pronuncian como [ı]: 'funny ['fʌnı]; mini ['mını].</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Ii, Yy у bu [ı]: 'funny ['fʌnı]; mini ['mını].</t>
+          <t>Ii, Yy у ненаголошеному складі читаються як [ı]: 'funny ['fʌnı]; mini ['mını].</t>
         </is>
       </c>
     </row>
@@ -82877,12 +82877,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Буква о в буквосочетаниях old ost olt читается как [əʊ]: old [əʊld ]; most [məʊst]; bolt [bəʊlt].</t>
+          <t>Буква о в буквосочетаниях old ost olt читается как [əʊ]: old [əʊld]; most [məʊst]; bolt [bəʊlt].</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>The letter o in the letter combinations old ost olt is pronounced [əʊ]: old [əʊld ]; most [məʊst]; bolt [bəʊlt].</t>
+          <t>The letter o in the letter combinations old ost olt is pronounced [əʊ]: old [əʊld]; most [məʊst]; bolt [bəʊlt].</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -82892,7 +82892,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Літера o у буквосполученнях old ost olt вимовляється як [əʊ]: old [əʊld ]; most [məʊst]; bolt [bəʊlt].</t>
+          <t>Літера o у буквосполученнях old ost olt вимовляється як [əʊ]: old [əʊld]; most [məʊst]; bolt [bəʊlt].</t>
         </is>
       </c>
     </row>
@@ -83052,12 +83052,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Буквосочетание tion  читается как [ʃ(ə)n]: 'action ]'ækʃ(ə)n]. Буквосочетание ture читается как [tʃə]: 'nature ['neıtʃə].</t>
+          <t>Буквосочетание tion  читается как [ʃ(ə)n]: 'action ['ækʃ(ə)n]. Буквосочетание ture читается как [tʃə]: 'nature ['neıtʃə].</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>The letter combination tion is read as [ʃ(ə)n]: 'action ]'ækʃ(ə)n]. The letter combination ture is read as [tʃə]: 'nature ['neıtʃə].</t>
+          <t>The letter combination tion is read as [ʃ(ə)n]: 'action ['ækʃ(ə)n]. The letter combination ture is read as [tʃə]: 'nature ['neıtʃə].</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -83067,7 +83067,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Буквосполучення tion читається як [ʃ(ə)n]: 'action ]'ækʃ(ə)n]. Буквосполучення ture читається як [tʃə]: 'nature ['neıtʃə].</t>
+          <t>Буквосполучення tion читається як [ʃ(ə)n]: 'action ['ækʃ(ə)n]. Буквосполучення ture читається як [tʃə]: 'nature ['neıtʃə].</t>
         </is>
       </c>
     </row>

</xml_diff>